<commit_message>
the prediction runs the model.
</commit_message>
<xml_diff>
--- a/Alert prediction data_frem.xlsx
+++ b/Alert prediction data_frem.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a72dd14889608c0/Desktop/NCV/datasets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a72dd14889608c0/Desktop/NCV/project code/ml model/lstm_scorepred/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1" documentId="8_{A41FB2EE-69BB-4AA7-ABC7-EE3742900E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C51A681-C52C-4D62-9159-46C28F629C46}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AD7807A2-C0C6-444D-BCA3-095AC47222FC}"/>
+    <workbookView minimized="1" xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" xr2:uid="{AD7807A2-C0C6-444D-BCA3-095AC47222FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>